<commit_message>
feat(content): refresh MB Bank account guide
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
@@ -5308,18 +5308,24 @@
       <x:c r="K5" s="22" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="L5" s="22" t="str">
-        <x:v>Ready</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L5" s="22" t="str">
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="M5" s="22" t="str">
         <x:v>Initial backlog / Item 1</x:v>
       </x:c>
-      <x:c r="N5" s="22"/>
-      <x:c r="O5" s="22"/>
-      <x:c r="P5" s="22"/>
-      <x:c r="Q5" s="22"/>
-      <x:c r="R5" s="22" t="str">
-        <x:v>Core acquisition</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N5" s="22" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O5" s="22" t="str">
+        <x:v>https://1phutdangky.com/mo-tai-khoan/mo-tai-khoan-mb-bank-online/</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P5" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q5" s="22" t="str">
+        <x:v>Pending push and existing Cloudflare deployment</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R5" s="22" t="str">
+        <x:v>Retained seeded first eligible P0 item. Updated existing account owner, not referral/card pages. Preserve approved title ending online, exact OneLink and MBAT113. No fixed reward claims or unpublished-route links.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10437,61 +10443,61 @@
       <x:c r="A5" t="str">
         <x:v>Next Queue #</x:v>
       </x:c>
-      <x:c r="B5" t="n">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B5" t="n">
         <x:f>IFERROR(INDEX('Evergreen Queue'!$A$5:$A$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)),"DISCOVERY")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
         <x:v>Next Asset ID</x:v>
       </x:c>
-      <x:c r="B6" t="str">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B6" t="str">
         <x:f>IF(B5="DISCOVERY","DISCOVERY",INDEX('Evergreen Queue'!$B$5:$B$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>A-PILLAR</x:v>
+        <x:v>R-PILLAR</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
         <x:v>Topic / Task</x:v>
       </x:c>
-      <x:c r="B7" t="str">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B7" t="str">
         <x:f>IF(B5="DISCOVERY","Run Discovery Mode",INDEX('Evergreen Queue'!$C$5:$C$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Update: Mở tài khoản MB Bank online</x:v>
+        <x:v>Publish: Mã giới thiệu MB Bank MBAT113</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
         <x:v>Cluster</x:v>
       </x:c>
-      <x:c r="B8" t="str">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B8" t="str">
         <x:f>IF(B5="DISCOVERY","All",INDEX('Evergreen Queue'!$D$5:$D$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Account</x:v>
+        <x:v>Referral</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
         <x:v>Work mode</x:v>
       </x:c>
-      <x:c r="B9" t="str">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B9" t="str">
         <x:f>IF(B5="DISCOVERY","Research",INDEX('Evergreen Queue'!$F$5:$F$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Update existing</x:v>
+        <x:v>New article</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
         <x:v>Canonical / Parent</x:v>
       </x:c>
-      <x:c r="B10" t="str">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B10" t="str">
         <x:f>IF(B5="DISCOVERY","Evergreen Queue",INDEX('Evergreen Queue'!$H$5:$H$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Pillar A</x:v>
+        <x:v>Pillar R</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="B11" t="str">
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B11" t="str">
         <x:f>IF(B5="DISCOVERY","P0",INDEX('Evergreen Queue'!$K$5:$K$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
         <x:v>P0</x:v>
       </x:c>
@@ -10714,22 +10720,52 @@
       <x:c r="A4" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B4" s="22"/>
-      <x:c r="C4" s="22"/>
-      <x:c r="D4" s="22"/>
-      <x:c r="E4" s="22"/>
-      <x:c r="F4" s="22"/>
-      <x:c r="G4" s="22"/>
-      <x:c r="H4" s="22"/>
-      <x:c r="I4" s="22"/>
-      <x:c r="J4" s="22"/>
-      <x:c r="K4" s="22"/>
-      <x:c r="L4" s="22"/>
-      <x:c r="M4" s="22"/>
-      <x:c r="N4" s="22"/>
-      <x:c r="O4" s="22"/>
-      <x:c r="P4" s="22"/>
-      <x:c r="Q4" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B4" s="22" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C4" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D4" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="E4" s="22" t="str">
+        <x:v>A-PILLAR</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="F4" s="22" t="str">
+        <x:v>Update: Mở tài khoản MB Bank online</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="G4" s="22" t="str">
+        <x:v>Update existing canonical; retain seed order, owner title ending online, MBAT113 and exact approved OneLink. No unpublished referral/card links.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="H4" s="22" t="str">
+        <x:v>https://1phutdangky.com/mo-tai-khoan/mo-tai-khoan-mb-bank-online/</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I4" s="22" t="str">
+        <x:v>2026-10-28: S1 official account guide (12/10/2026), rendered in Chrome; S2 MB247 contact; official App page rendered; account terms/eMB terms and 2026 individual fee PDF; MB News contact rendered. Original fee PDF visually checked page 1: ordinary account open/close free, 50,000 VND minimum balance. Approved OneLink checked for iOS app id1205807363 and Android app/store dispatcher. Existing owner-provided code MBAT113 retained; no new reward/age threshold asserted.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J4" s="22" t="str">
+        <x:v>src/content/articles/mo-tai-khoan/mo-tai-khoan-mb-bank-online.mdx; src/data/products/bank-accounts/mb-bank-account.json; docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K4" s="22" t="str">
+        <x:v>PASS npm run check (Astro build, Pagefind, validator): 20 HTML, 18 sitemap URLs. PASS git diff --check. Local Chrome: 375/390/768/1440 light/dark; canonical, metadata, JSON-LD, 3 identical OneLink CTAs, MBAT113 clipboard, consent denied/granted click/copy gating, no page errors/overflow. No separate lint/typecheck/test scripts. Workbook formulas recalculated and native features preserved.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L4" s="22" t="str">
+        <x:v>Pending content commit</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M4" s="22" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N4" s="22" t="str">
+        <x:v>Existing automatic Cloudflare Pages Git workflow</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O4" s="22" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P4" s="22" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q4" s="22" t="str">
+        <x:v>Updated A-PILLAR only. Referral/card pages not yet published, so bridge stays a short section in account article and no links to future owners. OneLink, reward-neutral stance and UI preserved.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="22" t="n">
@@ -18627,8 +18663,8 @@
       <x:c r="C5" s="22" t="str">
         <x:v>SEO Title</x:v>
       </x:c>
-      <x:c r="D5" s="22" t="str">
-        <x:v>Mở tài khoản MB Bank online: Cách đăng ký trên App MBBank</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D5" s="22" t="str">
+        <x:v>Hướng dẫn mở tài khoản MB Bank online</x:v>
       </x:c>
       <x:c r="E5" s="22" t="str">
         <x:v>177 Account/Generic seeds</x:v>
@@ -18666,8 +18702,8 @@
       <x:c r="P5" s="22" t="str">
         <x:v>Keep URL</x:v>
       </x:c>
-      <x:c r="Q5" s="22" t="str">
-        <x:v>Referral prominent in body.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q5" s="22" t="str">
+        <x:v>Giữ URL và tiêu đề chủ website đã chốt, online ở cuối.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -18680,8 +18716,8 @@
       <x:c r="C6" s="22" t="str">
         <x:v>H1</x:v>
       </x:c>
-      <x:c r="D6" s="22" t="str">
-        <x:v>Mở tài khoản MB Bank online: Cách đăng ký, điều kiện và mã giới thiệu</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D6" s="22" t="str">
+        <x:v>Hướng dẫn mở tài khoản MB Bank online</x:v>
       </x:c>
       <x:c r="E6" s="22" t="str">
         <x:v>Account + affiliate</x:v>
@@ -19693,11 +19729,11 @@
       <x:c r="B5" s="22" t="str">
         <x:v>Hot</x:v>
       </x:c>
-      <x:c r="C5" s="22" t="str">
-        <x:v>Mở tài khoản MB trên App</x:v>
-      </x:c>
-      <x:c r="D5" s="22" t="str">
-        <x:v>Xem cách dùng mã MBAT113</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C5" s="22" t="str">
+        <x:v>Mở App MBBank</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D5" s="22" t="str">
+        <x:v>Xem cách dùng mã MBAT113 trong bài; chuyển sang R-PILLAR khi URL đó đã xuất bản</x:v>
       </x:c>
       <x:c r="E5" s="22" t="str">
         <x:v>High</x:v>
@@ -19717,8 +19753,8 @@
       <x:c r="J5" s="22" t="str">
         <x:v>Không hứa reward</x:v>
       </x:c>
-      <x:c r="K5" s="22" t="str">
-        <x:v>cta_mb_account_open; click_mb_referral_guide</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K5" s="22" t="str">
+        <x:v>affiliate_click; referral_code_copy (existing consent-aware events)</x:v>
       </x:c>
       <x:c r="L5" s="22" t="str">
         <x:v>CTA → outbound</x:v>
@@ -20266,8 +20302,8 @@
       <x:c r="H5" s="22" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="I5" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I5" s="22" t="str">
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="J5" s="22" t="str">
         <x:v>Before publish</x:v>
@@ -20304,8 +20340,8 @@
       <x:c r="H6" s="22" t="str">
         <x:v>Low</x:v>
       </x:c>
-      <x:c r="I6" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I6" s="22" t="str">
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
         <x:v>If support details change</x:v>
@@ -20418,8 +20454,8 @@
       <x:c r="H9" s="22" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="I9" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I9" s="22" t="str">
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="J9" s="22" t="str">
         <x:v>Before publish</x:v>
@@ -20456,8 +20492,8 @@
       <x:c r="H10" s="22" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="I10" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I10" s="22" t="str">
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="J10" s="22" t="str">
         <x:v>Whenever affiliate setup changes</x:v>

</xml_diff>

<commit_message>
chore(content): record MB Bank production verification
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
@@ -5309,7 +5309,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L5" s="22" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M5" s="22" t="str">
         <x:v>Initial backlog / Item 1</x:v>
@@ -5320,9 +5320,11 @@
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O5" s="22" t="str">
         <x:v>https://1phutdangky.com/mo-tai-khoan/mo-tai-khoan-mb-bank-online/</x:v>
       </x:c>
-      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P5" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P5" s="22" t="str">
+        <x:v>18ec8141c1e7e44ba7b641b9c8e4f7745d57130b</x:v>
+      </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q5" s="22" t="str">
-        <x:v>Pending push and existing Cloudflare deployment</x:v>
+        <x:v>Cloudflare Pages success 9f4c41dc-4d09-4390-8e8a-4a600e7d17b1; production verified 2026-10-28</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R5" s="22" t="str">
         <x:v>Retained seeded first eligible P0 item. Updated existing account owner, not referral/card pages. Preserve approved title ending online, exact OneLink and MBAT113. No fixed reward claims or unpublished-route links.</x:v>
@@ -10723,7 +10725,9 @@
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B4" s="22" t="str">
         <x:v>2026-10-28</x:v>
       </x:c>
-      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C4" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C4" s="22" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D4" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -10749,19 +10753,19 @@
         <x:v>PASS npm run check (Astro build, Pagefind, validator): 20 HTML, 18 sitemap URLs. PASS git diff --check. Local Chrome: 375/390/768/1440 light/dark; canonical, metadata, JSON-LD, 3 identical OneLink CTAs, MBAT113 clipboard, consent denied/granted click/copy gating, no page errors/overflow. No separate lint/typecheck/test scripts. Workbook formulas recalculated and native features preserved.</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L4" s="22" t="str">
-        <x:v>Pending content commit</x:v>
+        <x:v>18ec8141c1e7e44ba7b641b9c8e4f7745d57130b</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M4" s="22" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Content pushed to origin/main; GitHub SHA verified</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N4" s="22" t="str">
-        <x:v>Existing automatic Cloudflare Pages Git workflow</x:v>
+        <x:v>Cloudflare Pages success 9f4c41dc-4d09-4390-8e8a-4a600e7d17b1 via existing Git integration</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O4" s="22" t="str">
-        <x:v>Pending</x:v>
+        <x:v>PASS production HTTP 200, canonical/title/meta/schema/sitemap, 3 exact CTAs, MBAT113 copy, consent gating, 375/390/768/1440 light/dark and no runtime errors/overflow</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P4" s="22" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q4" s="22" t="str">
         <x:v>Updated A-PILLAR only. Referral/card pages not yet published, so bridge stays a short section in account article and no links to future owners. OneLink, reward-neutral stance and UI preserved.</x:v>

</xml_diff>

<commit_message>
feat(content): publish MB Bank referral guide
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
@@ -5364,18 +5364,24 @@
       <x:c r="K6" s="22" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="L6" s="22" t="str">
-        <x:v>Ready</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L6" s="22" t="str">
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="M6" s="22" t="str">
         <x:v>Initial backlog / Item 2</x:v>
       </x:c>
-      <x:c r="N6" s="22"/>
-      <x:c r="O6" s="22"/>
-      <x:c r="P6" s="22"/>
-      <x:c r="Q6" s="22"/>
-      <x:c r="R6" s="22" t="str">
-        <x:v>Primary conversion</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N6" s="22" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O6" s="22" t="str">
+        <x:v>https://1phutdangky.com/ma-gioi-thieu-mb-bank/</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P6" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q6" s="22" t="str">
+        <x:v>Pending push and existing Cloudflare deployment</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R6" s="22" t="str">
+        <x:v>Published referral owner intent separately from Account; exact MBAT113 and approved OneLink reused. Official public guide field label verified; no fixed current screen order, autofill or reward guarantee. Official 2025 enrollment terms expired; payout date 2026 is not enrollment extension.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10447,7 +10453,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B5" t="n">
         <x:f>IFERROR(INDEX('Evergreen Queue'!$A$5:$A$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)),"DISCOVERY")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10456,7 +10462,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B6" t="str">
         <x:f>IF(B5="DISCOVERY","DISCOVERY",INDEX('Evergreen Queue'!$B$5:$B$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>R-PILLAR</x:v>
+        <x:v>A-ERRORS</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10465,7 +10471,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B7" t="str">
         <x:f>IF(B5="DISCOVERY","Run Discovery Mode",INDEX('Evergreen Queue'!$C$5:$C$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Publish: Mã giới thiệu MB Bank MBAT113</x:v>
+        <x:v>Publish: Không đăng ký được MB Bank</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -10474,7 +10480,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B8" t="str">
         <x:f>IF(B5="DISCOVERY","All",INDEX('Evergreen Queue'!$D$5:$D$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Referral</x:v>
+        <x:v>Account</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10492,7 +10498,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B10" t="str">
         <x:f>IF(B5="DISCOVERY","Evergreen Queue",INDEX('Evergreen Queue'!$H$5:$H$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Pillar R</x:v>
+        <x:v>A-ERRORS</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -10775,22 +10781,52 @@
       <x:c r="A5" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B5" s="22"/>
-      <x:c r="C5" s="22"/>
-      <x:c r="D5" s="22"/>
-      <x:c r="E5" s="22"/>
-      <x:c r="F5" s="22"/>
-      <x:c r="G5" s="22"/>
-      <x:c r="H5" s="22"/>
-      <x:c r="I5" s="22"/>
-      <x:c r="J5" s="22"/>
-      <x:c r="K5" s="22"/>
-      <x:c r="L5" s="22"/>
-      <x:c r="M5" s="22"/>
-      <x:c r="N5" s="22"/>
-      <x:c r="O5" s="22"/>
-      <x:c r="P5" s="22"/>
-      <x:c r="Q5" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B5" s="22" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C5" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D5" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="E5" s="22" t="str">
+        <x:v>R-PILLAR</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="F5" s="22" t="str">
+        <x:v>Publish: Mã giới thiệu MB Bank MBAT113</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="G5" s="22" t="str">
+        <x:v>New referral owner /ma-gioi-thieu-mb-bank/; preserve seeded order; account owner retains opening/fees intent. Verify source gate before publishing.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="H5" s="22" t="str">
+        <x:v>https://1phutdangky.com/ma-gioi-thieu-mb-bank/</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I5" s="22" t="str">
+        <x:v>2026-10-28: rendered official MB referral programme page and read linked 2025 T&amp;C PDF; enrollment ends 2025-12-31, payout ends 2026-12-31, no current reward claimed. Inspected official legacy guide image for optional referral section / Mã người giới thiệu (Mã RM); no assertion of exact current UI sequence. Official MB247 contact rendered. Owned MBAT113 setup retained. Exact OneLink dispatcher tested with iOS and Android UAs: expected app/store targets, no automatic attribution asserted.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J5" s="22" t="str">
+        <x:v>src/content/articles/ma-gioi-thieu-mb-bank.mdx; src/content/articles/ma-gioi-thieu-mb-bank-cover.png; src/content/articles/mo-tai-khoan/mo-tai-khoan-mb-bank-online.mdx; docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K5" s="22" t="str">
+        <x:v>PASS npm run check: Astro build + Pagefind + validator, 21 HTML /19 sitemap URLs. PASS git diff --check. Local Chrome 375/390/768/1440 light/dark, one H1, canonical, robots, BreadcrumbList, 3 exact OneLink CTAs, MBAT113 clipboard, consent-aware events, no overflow/runtime errors. Independent editorial/SEO source review: no actionable findings. No separate lint/typecheck/test scripts. Workbook recalculated; original native formatting/formulas preserved.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L5" s="22" t="str">
+        <x:v>Pending content commit</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M5" s="22" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N5" s="22" t="str">
+        <x:v>Existing automatic GitHub/Cloudflare Pages workflow</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O5" s="22" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P5" s="22" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q5" s="22" t="str">
+        <x:v>Queue #2 only; new referral owner plus minimal Account bridge link. No new current fee, age or reward claims. Distinct sections cover code, link, optionality as shown in published guide, benefit verification and forgotten/invalid code support. No extra FAQ or new support URLs.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="22" t="n">
@@ -18826,8 +18862,8 @@
       <x:c r="C8" s="22" t="str">
         <x:v>SEO Title</x:v>
       </x:c>
-      <x:c r="D8" s="22" t="str">
-        <x:v>Mã giới thiệu MB Bank MBAT113: Nhập ở đâu, dùng thế nào?</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D8" s="22" t="str">
+        <x:v>Mã giới thiệu MB Bank MBAT113: Cách dùng khi đăng ký online</x:v>
       </x:c>
       <x:c r="E8" s="22" t="str">
         <x:v>Referral money intent</x:v>
@@ -18865,8 +18901,8 @@
       <x:c r="P8" s="22" t="str">
         <x:v>Publish</x:v>
       </x:c>
-      <x:c r="Q8" s="22" t="str">
-        <x:v>Money page.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q8" s="22" t="str">
+        <x:v>Giữ tiêu đề kết thúc bằng online theo yêu cầu chủ website.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -18879,8 +18915,8 @@
       <x:c r="C9" s="22" t="str">
         <x:v>H1</x:v>
       </x:c>
-      <x:c r="D9" s="22" t="str">
-        <x:v>Mã giới thiệu MB Bank MBAT113: Cách dùng, nhập ở đâu và các lưu ý</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D9" s="22" t="str">
+        <x:v>Mã giới thiệu MB Bank MBAT113: Cách dùng khi đăng ký online</x:v>
       </x:c>
       <x:c r="E9" s="22" t="str">
         <x:v>Referral + questions</x:v>
@@ -18918,8 +18954,8 @@
       <x:c r="P9" s="22" t="str">
         <x:v>Required</x:v>
       </x:c>
-      <x:c r="Q9" s="22" t="str">
-        <x:v>Use MBAT113 only.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q9" s="22" t="str">
+        <x:v>Use MBAT113 only; link existing Account owner; unpublished support routes remain sections.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -18932,8 +18968,8 @@
       <x:c r="C10" s="22" t="str">
         <x:v>Answer block</x:v>
       </x:c>
-      <x:c r="D10" s="22" t="str">
-        <x:v>MBAT113 là mã giới thiệu được 1 Phút Đăng Ký sử dụng trong luồng đăng ký MB. Cách mã được nhập hoặc ghi nhận có thể thay đổi theo phiên bản App/link; hãy kiểm tra hướng dẫn và ngày kiểm chứng trước khi tiếp tục.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D10" s="22" t="str">
+        <x:v>MBAT113 là mã giới thiệu được 1 Phút Đăng Ký sử dụng khi hướng dẫn đăng ký App MBBank. Bạn nhập mã vào phần thông tin người giới thiệu trong ứng dụng và kiểm tra lại trước khi hoàn tất đăng ký. Quyền lợi phụ thuộc thể lệ MB áp dụng cho lượt đăng ký của bạn.</x:v>
       </x:c>
       <x:c r="E10" s="22" t="str">
         <x:v>Referral definition</x:v>
@@ -18971,8 +19007,8 @@
       <x:c r="P10" s="22" t="str">
         <x:v>Required</x:v>
       </x:c>
-      <x:c r="Q10" s="22" t="str">
-        <x:v>Exact code MBAT113.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q10" s="22" t="str">
+        <x:v>Owned code setup + publicly published guide label; legacy guide not proof of fixed current App sequence. No autofill/reward promise.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -19737,7 +19773,7 @@
         <x:v>Mở App MBBank</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D5" s="22" t="str">
-        <x:v>Xem cách dùng mã MBAT113 trong bài; chuyển sang R-PILLAR khi URL đó đã xuất bản</x:v>
+        <x:v>Xem cách dùng mã MBAT113 tại /ma-gioi-thieu-mb-bank/</x:v>
       </x:c>
       <x:c r="E5" s="22" t="str">
         <x:v>High</x:v>
@@ -19774,8 +19810,8 @@
       <x:c r="B6" s="22" t="str">
         <x:v>Very hot</x:v>
       </x:c>
-      <x:c r="C6" s="22" t="str">
-        <x:v>Dùng link đăng ký + mã MBAT113</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C6" s="22" t="str">
+        <x:v>Mở App MBBank</x:v>
       </x:c>
       <x:c r="D6" s="22" t="str">
         <x:v>Xem hướng dẫn mở tài khoản</x:v>
@@ -19798,8 +19834,8 @@
       <x:c r="J6" s="22" t="str">
         <x:v>Không urgency giả / reward unverified</x:v>
       </x:c>
-      <x:c r="K6" s="22" t="str">
-        <x:v>cta_mb_referral; outbound_mb_referral</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K6" s="22" t="str">
+        <x:v>affiliate_click; referral_code_copy (existing consent-aware events)</x:v>
       </x:c>
       <x:c r="L6" s="22" t="str">
         <x:v>Outbound / conversion</x:v>
@@ -20534,8 +20570,8 @@
       <x:c r="H11" s="22" t="str">
         <x:v>Very High</x:v>
       </x:c>
-      <x:c r="I11" s="22" t="str">
-        <x:v>2026-10-27</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I11" s="22" t="str">
+        <x:v>2026-10-28</x:v>
       </x:c>
       <x:c r="J11" s="22" t="str">
         <x:v>Every referral-benefit update</x:v>
@@ -20543,8 +20579,8 @@
       <x:c r="K11" s="22" t="str">
         <x:v>Mandatory for reward amount</x:v>
       </x:c>
-      <x:c r="L11" s="22" t="str">
-        <x:v>If unavailable, use neutral wording.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L11" s="22" t="str">
+        <x:v>Checked official referral page and linked /resources/files/2025/Referral-2025/tnc-referral-2025-(nfc).pdf: enrollment 2025-01-01 to 2025-12-31, payout end 2026-12-31. Historical evidence only; no current reward amount verified. Public guide label inspected; no fixed current screen order claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">

</xml_diff>

<commit_message>
chore(content): record MB Bank referral production verification
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
@@ -5365,7 +5365,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L6" s="22" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M6" s="22" t="str">
         <x:v>Initial backlog / Item 2</x:v>
@@ -5376,9 +5376,11 @@
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O6" s="22" t="str">
         <x:v>https://1phutdangky.com/ma-gioi-thieu-mb-bank/</x:v>
       </x:c>
-      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P6" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P6" s="22" t="str">
+        <x:v>23e10975c25df04a40a0910f59d7204809ebfa54</x:v>
+      </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q6" s="22" t="str">
-        <x:v>Pending push and existing Cloudflare deployment</x:v>
+        <x:v>Cloudflare Pages success 87b9ce08-3fa2-41ac-8d9b-d23e9f817f6f; production verified 2026-10-28</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R6" s="22" t="str">
         <x:v>Published referral owner intent separately from Account; exact MBAT113 and approved OneLink reused. Official public guide field label verified; no fixed current screen order, autofill or reward guarantee. Official 2025 enrollment terms expired; payout date 2026 is not enrollment extension.</x:v>
@@ -10784,7 +10786,9 @@
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B5" s="22" t="str">
         <x:v>2026-10-28</x:v>
       </x:c>
-      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C5" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C5" s="22" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D5" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -10810,19 +10814,19 @@
         <x:v>PASS npm run check: Astro build + Pagefind + validator, 21 HTML /19 sitemap URLs. PASS git diff --check. Local Chrome 375/390/768/1440 light/dark, one H1, canonical, robots, BreadcrumbList, 3 exact OneLink CTAs, MBAT113 clipboard, consent-aware events, no overflow/runtime errors. Independent editorial/SEO source review: no actionable findings. No separate lint/typecheck/test scripts. Workbook recalculated; original native formatting/formulas preserved.</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L5" s="22" t="str">
-        <x:v>Pending content commit</x:v>
+        <x:v>23e10975c25df04a40a0910f59d7204809ebfa54</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M5" s="22" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pushed to origin/main; GitHub SHA verified</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N5" s="22" t="str">
-        <x:v>Existing automatic GitHub/Cloudflare Pages workflow</x:v>
+        <x:v>Cloudflare Pages success 87b9ce08-3fa2-41ac-8d9b-d23e9f817f6f via existing Git integration</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O5" s="22" t="str">
-        <x:v>Pending</x:v>
+        <x:v>PASS production HTTP 200; one H1, metadata/OG image, canonical, Article/BreadcrumbList, sitemap exactly once (19 URLs), homepage/category discovery, reciprocal Account links, 3 exact CTAs, MBAT113 copy, consent gating, 375/390/768/1440 light/dark, no overflow/runtime errors</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P5" s="22" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q5" s="22" t="str">
         <x:v>Queue #2 only; new referral owner plus minimal Account bridge link. No new current fee, age or reward claims. Distinct sections cover code, link, optionality as shown in published guide, benefit verification and forgotten/invalid code support. No extra FAQ or new support URLs.</x:v>

</xml_diff>

<commit_message>
feat(content): publish MB Bank signup troubleshooting guide
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
@@ -5420,18 +5420,24 @@
       <x:c r="K7" s="22" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="L7" s="22" t="str">
-        <x:v>Ready</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L7" s="22" t="str">
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="M7" s="22" t="str">
         <x:v>Initial backlog / Item 3</x:v>
       </x:c>
-      <x:c r="N7" s="22"/>
-      <x:c r="O7" s="22"/>
-      <x:c r="P7" s="22"/>
-      <x:c r="Q7" s="22"/>
-      <x:c r="R7" s="22" t="str">
-        <x:v>Task completion</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N7" s="22" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O7" s="22" t="str">
+        <x:v>https://1phutdangky.com/khong-dang-ky-duoc-mb-bank/</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P7" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q7" s="22" t="str">
+        <x:v>Pending push and existing Cloudflare deployment</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R7" s="22" t="str">
+        <x:v>Queue #3 only. New support hub covers OTP/camera/eKYC/NFC/existing information/App interruption; Account keeps brief bridge. Reuse UI; no top product card or sticky CTA. One shared affiliate action after solutions and MB247, near shared disclosure. No fixed error-code causes, retry timers or approval/reward claims.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -10455,7 +10461,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B5" t="n">
         <x:f>IFERROR(INDEX('Evergreen Queue'!$A$5:$A$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)),"DISCOVERY")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10464,7 +10470,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B6" t="str">
         <x:f>IF(B5="DISCOVERY","DISCOVERY",INDEX('Evergreen Queue'!$B$5:$B$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>A-ERRORS</x:v>
+        <x:v>A-NEED</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10473,7 +10479,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B7" t="str">
         <x:f>IF(B5="DISCOVERY","Run Discovery Mode",INDEX('Evergreen Queue'!$C$5:$C$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Publish: Không đăng ký được MB Bank</x:v>
+        <x:v>Publish: Mở tài khoản MB Bank cần gì?</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -10500,7 +10506,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B10" t="str">
         <x:f>IF(B5="DISCOVERY","Evergreen Queue",INDEX('Evergreen Queue'!$H$5:$H$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>A-ERRORS</x:v>
+        <x:v>A-NEED</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -10509,7 +10515,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B11" t="str">
         <x:f>IF(B5="DISCOVERY","P0",INDEX('Evergreen Queue'!$K$5:$K$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -10836,22 +10842,52 @@
       <x:c r="A6" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B6" s="22"/>
-      <x:c r="C6" s="22"/>
-      <x:c r="D6" s="22"/>
-      <x:c r="E6" s="22"/>
-      <x:c r="F6" s="22"/>
-      <x:c r="G6" s="22"/>
-      <x:c r="H6" s="22"/>
-      <x:c r="I6" s="22"/>
-      <x:c r="J6" s="22"/>
-      <x:c r="K6" s="22"/>
-      <x:c r="L6" s="22"/>
-      <x:c r="M6" s="22"/>
-      <x:c r="N6" s="22"/>
-      <x:c r="O6" s="22"/>
-      <x:c r="P6" s="22"/>
-      <x:c r="Q6" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B6" s="22" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C6" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D6" s="22" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="E6" s="22" t="str">
+        <x:v>A-ERRORS</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="F6" s="22" t="str">
+        <x:v>Publish: Không đăng ký được MB Bank</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="G6" s="22" t="str">
+        <x:v>New troubleshooting hub; retain seeded first eligible P0. Account retains registration/fees and Referral retains code intent; support article solves errors before affiliate action.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="H6" s="22" t="str">
+        <x:v>https://1phutdangky.com/khong-dang-ky-duoc-mb-bank/</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I6" s="22" t="str">
+        <x:v>2026-10-29: official https://www.mbbank.com.vn/Contact via web fetch (MB247 personal phones/email/support scope); MB-owned current AppStore id1205807363 and GooglePlay com.mbmobile listings. Apple camera permissions iph168c4bbd5 and SMS support118433; Google Android permissions9431959 and Messages9077245; Samsung nfc-not-working-samsung-galaxy-device. Direct rendered MB pages returned Access Denied; no authenticated App flow or arbitrary error-code diagnosis claimed. Exact approved OneLink tested with iOS/Android UAs: 200 app/store dispatchers. Shared MBAT113 offer/facts unchanged.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J6" s="22" t="str">
+        <x:v>src/content/articles/khong-dang-ky-duoc-mb-bank.mdx; src/content/articles/khong-dang-ky-duoc-mb-bank-cover.png; src/content/articles/mo-tai-khoan/mo-tai-khoan-mb-bank-online.mdx; docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K6" s="22" t="str">
+        <x:v>PASS npm run check (Astro build, Pagefind, validator):22 HTML/20 sitemap URLs. PASS git diff --check. Local Chrome375/390/768/1440 light/dark; one H1, canonical, Article/BreadcrumbList, OG image, TOC anchors, sitemap membership, discovery and reciprocal Account links; support before 1 exact OneLink CTA, disclosure before action, consent denied/granted events, no overflow/runtime errors. No separate lint/typecheck/test scripts. Workbook recalculated and native features preserved.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L6" s="22" t="str">
+        <x:v>Pending content commit</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M6" s="22" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N6" s="22" t="str">
+        <x:v>Existing automatic GitHub/Cloudflare Pages integration</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O6" s="22" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P6" s="22" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q6" s="22" t="str">
+        <x:v>New support URL with existing components. Affiliate UI is rendered once in body after assistance; no ProductCard/sticky sales action before error resolution. Registration guide retains account owner URL, title, code and exact OneLink; only error bridge and update date changed. A-OTP/A-EKYC/A-EXISTS and future A-NFC remain separate backlog items, not executed or marked Done in this run.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="22" t="n">
@@ -19078,8 +19114,8 @@
       <x:c r="C12" s="22" t="str">
         <x:v>SEO Title</x:v>
       </x:c>
-      <x:c r="D12" s="22" t="str">
-        <x:v>Không đăng ký được MB Bank: Các lỗi thường gặp và cách xử lý</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D12" s="22" t="str">
+        <x:v>Không đăng ký được MB Bank: Cách xử lý lỗi online</x:v>
       </x:c>
       <x:c r="E12" s="22" t="str">
         <x:v>Error umbrella</x:v>
@@ -19117,8 +19153,8 @@
       <x:c r="P12" s="22" t="str">
         <x:v>Publish</x:v>
       </x:c>
-      <x:c r="Q12" s="22" t="str">
-        <x:v>No sensitive data collection.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q12" s="22" t="str">
+        <x:v>Title ends online per owner. No unsupported numeric error mapping or exact current App screen flow. Existing reusable body CTA/disclosure after solutions and MB247; no shared component change.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -19937,11 +19973,11 @@
       <x:c r="B9" s="22" t="str">
         <x:v>Hot/problem</x:v>
       </x:c>
-      <x:c r="C9" s="22" t="str">
-        <x:v>Tiếp tục mở tài khoản sau khi xử lý</x:v>
-      </x:c>
-      <x:c r="D9" s="22" t="str">
-        <x:v>Xem MBAT113 nếu đang ở bước referral</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C9" s="22" t="str">
+        <x:v>Mở App MBBank (after solutions and MB247)</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D9" s="22" t="str">
+        <x:v>Contextual link to /ma-gioi-thieu-mb-bank/ for referral-specific issues</x:v>
       </x:c>
       <x:c r="E9" s="22" t="str">
         <x:v>Low-Medium</x:v>
@@ -19961,14 +19997,14 @@
       <x:c r="J9" s="22" t="str">
         <x:v>Không sales-first</x:v>
       </x:c>
-      <x:c r="K9" s="22" t="str">
-        <x:v>mb_error_to_account; mb_error_to_referral</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K9" s="22" t="str">
+        <x:v>affiliate_click (existing consent-aware event), position article-recovery</x:v>
       </x:c>
       <x:c r="L9" s="22" t="str">
         <x:v>Assisted conversion</x:v>
       </x:c>
-      <x:c r="M9" s="22" t="str">
-        <x:v>Task completion first.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M9" s="22" t="str">
+        <x:v>Support-first knowledge article; products[] empty and auto affiliate layout off. Shared AffiliateDisclosure + AffiliateCTA explicitly rendered once at end.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -20385,7 +20421,7 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I6" s="22" t="str">
-        <x:v>2026-10-28</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="J6" s="22" t="str">
         <x:v>If support details change</x:v>

</xml_diff>

<commit_message>
chore(content): record MB Bank troubleshooting production verification
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
@@ -5421,7 +5421,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L7" s="22" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M7" s="22" t="str">
         <x:v>Initial backlog / Item 3</x:v>
@@ -5432,9 +5432,11 @@
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O7" s="22" t="str">
         <x:v>https://1phutdangky.com/khong-dang-ky-duoc-mb-bank/</x:v>
       </x:c>
-      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P7" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P7" s="22" t="str">
+        <x:v>c6c1a23073d828e6028f9573f65af3c70eae0f3e</x:v>
+      </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q7" s="22" t="str">
-        <x:v>Pending push and existing Cloudflare deployment</x:v>
+        <x:v>Cloudflare Pages success 953b7adf-5f52-4156-9432-0acac84a8ad9; production verified 2026-10-29</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R7" s="22" t="str">
         <x:v>Queue #3 only. New support hub covers OTP/camera/eKYC/NFC/existing information/App interruption; Account keeps brief bridge. Reuse UI; no top product card or sticky CTA. One shared affiliate action after solutions and MB247, near shared disclosure. No fixed error-code causes, retry timers or approval/reward claims.</x:v>
@@ -10845,7 +10847,9 @@
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B6" s="22" t="str">
         <x:v>2026-10-29</x:v>
       </x:c>
-      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C6" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C6" s="22" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D6" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -10871,19 +10875,19 @@
         <x:v>PASS npm run check (Astro build, Pagefind, validator):22 HTML/20 sitemap URLs. PASS git diff --check. Local Chrome375/390/768/1440 light/dark; one H1, canonical, Article/BreadcrumbList, OG image, TOC anchors, sitemap membership, discovery and reciprocal Account links; support before 1 exact OneLink CTA, disclosure before action, consent denied/granted events, no overflow/runtime errors. No separate lint/typecheck/test scripts. Workbook recalculated and native features preserved.</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L6" s="22" t="str">
-        <x:v>Pending content commit</x:v>
+        <x:v>c6c1a23073d828e6028f9573f65af3c70eae0f3e</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M6" s="22" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pushed to origin/main; GitHub SHA verified</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N6" s="22" t="str">
-        <x:v>Existing automatic GitHub/Cloudflare Pages integration</x:v>
+        <x:v>Cloudflare Pages success 953b7adf-5f52-4156-9432-0acac84a8ad9 through existing Git integration</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O6" s="22" t="str">
-        <x:v>Pending</x:v>
+        <x:v>PASS production HTTP200; H1/metadata/OG image/canonical/Article/BreadcrumbList;20 sitemap URLs;TOC anchors;homepage/category/Account links;375/390/768/1440 light/dark;support-first single exact OneLink CTA and consent gating;no overflow/runtime errors;Account title/canonical/3 OneLinks unchanged</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P6" s="22" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q6" s="22" t="str">
         <x:v>New support URL with existing components. Affiliate UI is rendered once in body after assistance; no ProductCard/sticky sales action before error resolution. Registration guide retains account owner URL, title, code and exact OneLink; only error bridge and update date changed. A-OTP/A-EKYC/A-EXISTS and future A-NFC remain separate backlog items, not executed or marked Done in this run.</x:v>

</xml_diff>

<commit_message>
fix(content): align article URLs with their categories
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
@@ -833,8 +833,8 @@
       <x:c r="B8" s="22" t="str">
         <x:v>Business/affiliate expansion</x:v>
       </x:c>
-      <x:c r="C8" s="22" t="str">
-        <x:v>https://1phutdangky.com/ma-gioi-thieu-mb-bank/</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C8" s="22" t="str">
+        <x:v>https://1phutdangky.com/mo-tai-khoan/ma-gioi-thieu-mb-bank/</x:v>
       </x:c>
       <x:c r="D8" s="22" t="str">
         <x:v>Conversion pillar P0; mã dùng xuyên hệ thống: MBAT113.</x:v>
@@ -847,8 +847,8 @@
       <x:c r="B9" s="22" t="str">
         <x:v>34 keywords</x:v>
       </x:c>
-      <x:c r="C9" s="22" t="str">
-        <x:v>https://1phutdangky.com/mo-the-mb-bank-online/</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C9" s="22" t="str">
+        <x:v>https://1phutdangky.com/the-tin-dung/mo-the-mb-bank-online/</x:v>
       </x:c>
       <x:c r="D9" s="22" t="str">
         <x:v>Canonical owner của intent thẻ MB.</x:v>
@@ -1179,8 +1179,8 @@
       <x:c r="F6" s="22" t="str">
         <x:v>New article</x:v>
       </x:c>
-      <x:c r="G6" s="22" t="str">
-        <x:v>Create /ma-gioi-thieu-mb-bank/</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="G6" s="22" t="str">
+        <x:v>Create /mo-tai-khoan/ma-gioi-thieu-mb-bank/</x:v>
       </x:c>
       <x:c r="H6" s="22" t="str">
         <x:v>Pillar R</x:v>
@@ -5349,8 +5349,8 @@
       <x:c r="F6" s="22" t="str">
         <x:v>New article</x:v>
       </x:c>
-      <x:c r="G6" s="22" t="str">
-        <x:v>Create /ma-gioi-thieu-mb-bank/</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="G6" s="22" t="str">
+        <x:v>Create /mo-tai-khoan/ma-gioi-thieu-mb-bank/</x:v>
       </x:c>
       <x:c r="H6" s="22" t="str">
         <x:v>Pillar R</x:v>
@@ -5374,7 +5374,7 @@
         <x:v>2026-10-28</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O6" s="22" t="str">
-        <x:v>https://1phutdangky.com/ma-gioi-thieu-mb-bank/</x:v>
+        <x:v>https://1phutdangky.com/mo-tai-khoan/ma-gioi-thieu-mb-bank/</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P6" s="22" t="str">
         <x:v>23e10975c25df04a40a0910f59d7204809ebfa54</x:v>
@@ -5430,7 +5430,7 @@
         <x:v>2026-10-29</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O7" s="22" t="str">
-        <x:v>https://1phutdangky.com/khong-dang-ky-duoc-mb-bank/</x:v>
+        <x:v>https://1phutdangky.com/mo-tai-khoan/khong-dang-ky-duoc-mb-bank/</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P7" s="22" t="str">
         <x:v>c6c1a23073d828e6028f9573f65af3c70eae0f3e</x:v>
@@ -15807,8 +15807,8 @@
       <x:c r="A7" s="22" t="str">
         <x:v>Referral Pillar URL</x:v>
       </x:c>
-      <x:c r="B7" s="22" t="str">
-        <x:v>https://1phutdangky.com/ma-gioi-thieu-mb-bank/</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B7" s="22" t="str">
+        <x:v>https://1phutdangky.com/mo-tai-khoan/ma-gioi-thieu-mb-bank/</x:v>
       </x:c>
       <x:c r="C7" s="22" t="str">
         <x:v>URL</x:v>
@@ -15821,8 +15821,8 @@
       <x:c r="A8" s="22" t="str">
         <x:v>Card Pillar URL</x:v>
       </x:c>
-      <x:c r="B8" s="22" t="str">
-        <x:v>https://1phutdangky.com/mo-the-mb-bank-online/</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B8" s="22" t="str">
+        <x:v>https://1phutdangky.com/the-tin-dung/mo-the-mb-bank-online/</x:v>
       </x:c>
       <x:c r="C8" s="22" t="str">
         <x:v>URL</x:v>
@@ -17698,8 +17698,8 @@
       <x:c r="J6" s="22" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K6" s="22" t="str">
-        <x:v>/ma-gioi-thieu-mb-bank/</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K6" s="22" t="str">
+        <x:v>/mo-tai-khoan/ma-gioi-thieu-mb-bank/</x:v>
       </x:c>
       <x:c r="L6" s="22" t="str">
         <x:v>R↔A; R→R-support</x:v>
@@ -17985,8 +17985,8 @@
       <x:c r="J13" s="22" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K13" s="22" t="str">
-        <x:v>/mo-the-mb-bank-online/</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K13" s="22" t="str">
+        <x:v>/the-tin-dung/mo-the-mb-bank-online/</x:v>
       </x:c>
       <x:c r="L13" s="22" t="str">
         <x:v>C↔A</x:v>
@@ -19817,7 +19817,7 @@
         <x:v>Mở App MBBank</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D5" s="22" t="str">
-        <x:v>Xem cách dùng mã MBAT113 tại /ma-gioi-thieu-mb-bank/</x:v>
+        <x:v>Xem cách dùng mã MBAT113 tại /mo-tai-khoan/ma-gioi-thieu-mb-bank/</x:v>
       </x:c>
       <x:c r="E5" s="22" t="str">
         <x:v>High</x:v>
@@ -19981,7 +19981,7 @@
         <x:v>Mở App MBBank (after solutions and MB247)</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D9" s="22" t="str">
-        <x:v>Contextual link to /ma-gioi-thieu-mb-bank/ for referral-specific issues</x:v>
+        <x:v>Contextual link to /mo-tai-khoan/ma-gioi-thieu-mb-bank/ for referral-specific issues</x:v>
       </x:c>
       <x:c r="E9" s="22" t="str">
         <x:v>Low-Medium</x:v>

</xml_diff>

<commit_message>
feat(content): publish MB Bank account preparation guide
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
@@ -5476,18 +5476,24 @@
       <x:c r="K8" s="22" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="L8" s="22" t="str">
-        <x:v>Ready</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L8" s="22" t="str">
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="M8" s="22" t="str">
         <x:v>Initial backlog / Item 4</x:v>
       </x:c>
-      <x:c r="N8" s="22"/>
-      <x:c r="O8" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N8" s="22" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O8" s="22" t="str">
+        <x:v>https://1phutdangky.com/mo-tai-khoan/mo-tai-khoan-mb-bank-can-gi/</x:v>
+      </x:c>
       <x:c r="P8" s="22"/>
-      <x:c r="Q8" s="22"/>
-      <x:c r="R8" s="22" t="str">
-        <x:v>Qualification</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q8" s="22" t="str">
+        <x:v>Pending push and existing Cloudflare deployment</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R8" s="22" t="str">
+        <x:v>Queue #4 only. Preparation/eligibility checklist; Account owns how-to/fees, Referral owns MBAT113, troubleshooting stays in support hub. One internal Account action after readiness guidance; contextual Referral link. Current law and live MB-owned store/terms sources support claims; no authenticated App-flow claims. Shared title visual/social images generated at build, no new cover asset.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10463,7 +10469,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B5" t="n">
         <x:f>IFERROR(INDEX('Evergreen Queue'!$A$5:$A$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)),"DISCOVERY")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10472,7 +10478,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B6" t="str">
         <x:f>IF(B5="DISCOVERY","DISCOVERY",INDEX('Evergreen Queue'!$B$5:$B$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>A-NEED</x:v>
+        <x:v>A-AGE</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10481,7 +10487,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B7" t="str">
         <x:f>IF(B5="DISCOVERY","Run Discovery Mode",INDEX('Evergreen Queue'!$C$5:$C$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>Publish: Mở tài khoản MB Bank cần gì?</x:v>
+        <x:v>Publish: Bao nhiêu tuổi được mở tài khoản MB Bank?</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -10508,7 +10514,7 @@
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B10" t="str">
         <x:f>IF(B5="DISCOVERY","Evergreen Queue",INDEX('Evergreen Queue'!$H$5:$H$164,MATCH("Ready",'Evergreen Queue'!$L$5:$L$164,0)))</x:f>
-        <x:v>A-NEED</x:v>
+        <x:v>A-AGE</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -10897,22 +10903,52 @@
       <x:c r="A7" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B7" s="22"/>
-      <x:c r="C7" s="22"/>
-      <x:c r="D7" s="22"/>
-      <x:c r="E7" s="22"/>
-      <x:c r="F7" s="22"/>
-      <x:c r="G7" s="22"/>
-      <x:c r="H7" s="22"/>
-      <x:c r="I7" s="22"/>
-      <x:c r="J7" s="22"/>
-      <x:c r="K7" s="22"/>
-      <x:c r="L7" s="22"/>
-      <x:c r="M7" s="22"/>
-      <x:c r="N7" s="22"/>
-      <x:c r="O7" s="22"/>
-      <x:c r="P7" s="22"/>
-      <x:c r="Q7" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B7" s="22" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C7" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D7" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="E7" s="22" t="str">
+        <x:v>A-NEED</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="F7" s="22" t="str">
+        <x:v>Publish: Mở tài khoản MB Bank cần gì?</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="G7" s="22" t="str">
+        <x:v>New eligibility/preparation support article; first eligible seeded P1. Own checklist/requirements intent; Account retains registration/fees and Referral retains code intent.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="H7" s="22" t="str">
+        <x:v>https://1phutdangky.com/mo-tai-khoan/mo-tai-khoan-mb-bank-can-gi/</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I7" s="22" t="str">
+        <x:v>2026-10-29: MB S1 official account guide indexed text (dated2026-10-12); direct HTTP403/webfetch404 access constraint, not claimed live-page verification. Primary claims checked against official NHNN21/VBHN-NHNN consolidated17/2024+25/2025, Arts11/12/16 (PDF pp7-9,18-20); live200 MB eMB terms PDF, MB-owned AppStore id1205807363 and GooglePlay com.mbmobile (app identity/compatibility/contact); Apple camera and Samsung NFC device guidance. No authenticated current MB onboarding flow tested; no fixed screen sequence or universal NFC/VNeID alternative claimed.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="J7" s="22" t="str">
+        <x:v>src/content/articles/mo-tai-khoan/mo-tai-khoan-mb-bank-can-gi.mdx; src/content/articles/mo-tai-khoan/mo-tai-khoan-mb-bank-online.mdx; docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx. Social PNG generated automatically by existing build endpoint.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K7" s="22" t="str">
+        <x:v>PASS npm run check (Astro build, Pagefind, validator):23 HTML/21 sitemap URLs. PASS git diff --check. Local Chrome375/390/768/1440 light/dark: one H1, title/card/OG/Twitter image sync, canonical/Article/BreadcrumbList, TOC anchors, sitemap once, Pagefind search, homepage/category/Account discovery. Internal Account action after checklist and contextual Referral link. Account retains3 exact OneLinks, MBAT113 clipboard and denied/granted consent behavior. No page errors/overflow. Independent editorial/source review passed after resolving two unsupported assumptions. No separate lint/typecheck/test scripts. Workbook recalculated and native features preserved.</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L7" s="22" t="str">
+        <x:v>Pending content commit</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M7" s="22" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N7" s="22" t="str">
+        <x:v>Existing automatic GitHub/Cloudflare Pages integration</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O7" s="22" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P7" s="22" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q7" s="22" t="str">
+        <x:v>New standalone preparation URL; no full registration sequence, fee table or referral mechanics duplicated. Minimal Account bridge only. No product data, shared UI, analytics, DNS or deployment configuration changes. MB source-access constraint handled through accessible primary legal/MB-owned sources; indexed guide supporting only. A-AGE/A-NFC not executed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="22" t="n">
@@ -19171,8 +19207,8 @@
       <x:c r="C13" s="22" t="str">
         <x:v>SEO Title</x:v>
       </x:c>
-      <x:c r="D13" s="22" t="str">
-        <x:v>Mở tài khoản MB Bank cần gì? Điều kiện, giấy tờ và điện thoại cần chuẩn bị</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D13" s="22" t="str">
+        <x:v>Mở tài khoản MB Bank cần gì? Chuẩn bị để đăng ký online</x:v>
       </x:c>
       <x:c r="E13" s="22" t="str">
         <x:v>Preparation</x:v>
@@ -19210,8 +19246,8 @@
       <x:c r="P13" s="22" t="str">
         <x:v>Publish</x:v>
       </x:c>
-      <x:c r="Q13" s="22" t="str">
-        <x:v>Strong support.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q13" s="22" t="str">
+        <x:v>Title ends online. Own pre-registration readiness; brief Art11/16 eligibility, documents and device checks. Account/Referral internal links after answer; no top product card/sticky, no separate cover, no fixed App screens or cross-device OTP guarantee.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -20018,11 +20054,11 @@
       <x:c r="B10" s="22" t="str">
         <x:v>Warm</x:v>
       </x:c>
-      <x:c r="C10" s="22" t="str">
-        <x:v>Bắt đầu mở tài khoản MB</x:v>
-      </x:c>
-      <x:c r="D10" s="22" t="str">
-        <x:v>Xem mã MBAT113</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C10" s="22" t="str">
+        <x:v>Xem hướng dẫn mở tài khoản MB Bank</x:v>
+      </x:c>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D10" s="22" t="str">
+        <x:v>Xem cách dùng mã giới thiệu MBAT113</x:v>
       </x:c>
       <x:c r="E10" s="22" t="str">
         <x:v>Medium</x:v>
@@ -20042,14 +20078,14 @@
       <x:c r="J10" s="22" t="str">
         <x:v>Không nhồi CTA</x:v>
       </x:c>
-      <x:c r="K10" s="22" t="str">
-        <x:v>mb_need_to_account; mb_need_to_referral</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="K10" s="22" t="str">
+        <x:v>Existing consent-aware page_view; native internal links, no new click-event types</x:v>
       </x:c>
       <x:c r="L10" s="22" t="str">
         <x:v>Qualified click</x:v>
       </x:c>
-      <x:c r="M10" s="22" t="str">
-        <x:v>Preparation.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M10" s="22" t="str">
+        <x:v>Preparation article: one internal Account button after checklist/qualification at end, contextual Referral link. products[] empty; no auto product card/sticky or direct affiliate action.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -20387,7 +20423,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="I5" s="22" t="str">
-        <x:v>2026-10-28</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
       <x:c r="J5" s="22" t="str">
         <x:v>Before publish</x:v>
@@ -20395,8 +20431,8 @@
       <x:c r="K5" s="22" t="str">
         <x:v>Required for account/age claims</x:v>
       </x:c>
-      <x:c r="L5" s="22" t="str">
-        <x:v>Recheck current page.</x:v>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L5" s="22" t="str">
+        <x:v>2026-10-29: indexed official guide dated2026-10-12 available; direct request403/web404, access constraint not live verification. A-NEED eligibility/docs grounded in official NHNN21/VBHN-NHNN Art11/12/16, MB-owned live store listings and accessible eMB terms. Current App onboarding screens not tested. Recheck live provider sources before future age/flow claims.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">

</xml_diff>

<commit_message>
chore(content): record MB Bank preparation production verification
</commit_message>
<xml_diff>
--- a/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
+++ b/docs/content/1phutdangky_MB_Bank_Evergreen_Content_Engine.xlsx
@@ -5477,7 +5477,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L8" s="22" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M8" s="22" t="str">
         <x:v>Initial backlog / Item 4</x:v>
@@ -5488,9 +5488,11 @@
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O8" s="22" t="str">
         <x:v>https://1phutdangky.com/mo-tai-khoan/mo-tai-khoan-mb-bank-can-gi/</x:v>
       </x:c>
-      <x:c r="P8" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P8" s="22" t="str">
+        <x:v>568b6f81666008993da41faec9af2191662f4c4c</x:v>
+      </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q8" s="22" t="str">
-        <x:v>Pending push and existing Cloudflare deployment</x:v>
+        <x:v>Cloudflare Pages success 165445a9-1401-418a-9ad6-344ed6c0cb56; production verified 2026-10-29</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="R8" s="22" t="str">
         <x:v>Queue #4 only. Preparation/eligibility checklist; Account owns how-to/fees, Referral owns MBAT113, troubleshooting stays in support hub. One internal Account action after readiness guidance; contextual Referral link. Current law and live MB-owned store/terms sources support claims; no authenticated App-flow claims. Shared title visual/social images generated at build, no new cover asset.</x:v>
@@ -10906,7 +10908,9 @@
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="B7" s="22" t="str">
         <x:v>2026-10-29</x:v>
       </x:c>
-      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C7" s="22"/>
+      <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="C7" s="22" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="D7" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -10932,19 +10936,19 @@
         <x:v>PASS npm run check (Astro build, Pagefind, validator):23 HTML/21 sitemap URLs. PASS git diff --check. Local Chrome375/390/768/1440 light/dark: one H1, title/card/OG/Twitter image sync, canonical/Article/BreadcrumbList, TOC anchors, sitemap once, Pagefind search, homepage/category/Account discovery. Internal Account action after checklist and contextual Referral link. Account retains3 exact OneLinks, MBAT113 clipboard and denied/granted consent behavior. No page errors/overflow. Independent editorial/source review passed after resolving two unsupported assumptions. No separate lint/typecheck/test scripts. Workbook recalculated and native features preserved.</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="L7" s="22" t="str">
-        <x:v>Pending content commit</x:v>
+        <x:v>568b6f81666008993da41faec9af2191662f4c4c</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="M7" s="22" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pushed to origin/main; GitHub SHA verified</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="N7" s="22" t="str">
-        <x:v>Existing automatic GitHub/Cloudflare Pages integration</x:v>
+        <x:v>Cloudflare Pages success 165445a9-1401-418a-9ad6-344ed6c0cb56 through existing Git integration</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="O7" s="22" t="str">
-        <x:v>Pending</x:v>
+        <x:v>PASS production HTTP200; one H1, canonical/meta/Article/BreadcrumbList/OG/Twitter image sync;21 sitemap URLs and Pagefind;TOC anchors;homepage/category/Account bridge;375/390/768/1440 light/dark;internal Account action and Referral link after checklist;Account retains MBAT113 copy,3 exact OneLinks and denied/granted analytics consent;no overflow/runtime errors</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="P7" s="22" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="Q7" s="22" t="str">
         <x:v>New standalone preparation URL; no full registration sequence, fee table or referral mechanics duplicated. Minimal Account bridge only. No product data, shared UI, analytics, DNS or deployment configuration changes. MB source-access constraint handled through accessible primary legal/MB-owned sources; indexed guide supporting only. A-AGE/A-NFC not executed.</x:v>

</xml_diff>